<commit_message>
Update IT23335578_Assignment 1 - Test cases.xlsx
</commit_message>
<xml_diff>
--- a/IT23335578/IT23335578_Assignment 1 - Test cases.xlsx
+++ b/IT23335578/IT23335578_Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\SLIIT\Y3 S2 SLIIT\ITPM\test_automation\IT23335578\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\My Projects\IT23335578_ITPM_Assignment_1\IT23335578\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B24D14-E994-464D-AA30-3912A7B973CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E02F3AD-AADD-465D-9353-32BB08B376BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="247">
   <si>
     <t>TC ID</t>
   </si>
@@ -362,18 +362,9 @@
     <t>English Abbreviations/Acronyms in Singlish</t>
   </si>
   <si>
-    <t>Rationale: The input includes common English abbreviations or acronyms.</t>
-  </si>
-  <si>
     <t>Neg_0026</t>
   </si>
   <si>
-    <t>Mata oyage cv eka dala thiyanna</t>
-  </si>
-  <si>
-    <t>මට ඔයාගේ cv එක දාලා තියන්න</t>
-  </si>
-  <si>
     <t>Neg_0027</t>
   </si>
   <si>
@@ -386,9 +377,6 @@
     <t>English Clipped Forms in Singlish</t>
   </si>
   <si>
-    <t>Rationale: Shortened English word forms are used.</t>
-  </si>
-  <si>
     <t>Neg_0028</t>
   </si>
   <si>
@@ -407,9 +395,6 @@
     <t>Place Names Embedded in Singlish</t>
   </si>
   <si>
-    <t>Rationale: The input includes names of specific locations.</t>
-  </si>
-  <si>
     <t>Neg_0030</t>
   </si>
   <si>
@@ -431,9 +416,6 @@
     <t>Person Names Embedded in Singlish</t>
   </si>
   <si>
-    <t>Rationale: The input contains a specific person's name.</t>
-  </si>
-  <si>
     <t>Neg_0032</t>
   </si>
   <si>
@@ -527,9 +509,6 @@
     <t>Inputs with Dates</t>
   </si>
   <si>
-    <t>Rationale: The input includes date information.</t>
-  </si>
-  <si>
     <t>Neg_0040</t>
   </si>
   <si>
@@ -599,9 +578,6 @@
     <t>Online Indentifiers in Singlish</t>
   </si>
   <si>
-    <t>Rationale: The input contains handles or online identifiers.</t>
-  </si>
-  <si>
     <t>Neg_0046</t>
   </si>
   <si>
@@ -623,9 +599,6 @@
     <t>Inputs Containing Emojis</t>
   </si>
   <si>
-    <t>Rationale: The input includes graphical emojis.</t>
-  </si>
-  <si>
     <t>Neg_0048</t>
   </si>
   <si>
@@ -660,6 +633,147 @@
   </si>
   <si>
     <t>I need to do this quickly mch, because mt time ekka na bn</t>
+  </si>
+  <si>
+    <t>Rationale: The overall message is a question.  Evidence : "para pathtada yanne?"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "pathtada"</t>
+  </si>
+  <si>
+    <t>Rationale: The overall message is a question.  Evidence : "wde krl iwarda?"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "psidu"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale: The overall message is a command. </t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "ganth"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "dhn"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidense : " wasana wantha"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidense : "dhwalk"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "me ptha gnhn nimesh gn"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "denk"</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains numerical values. Evidence : "100 denk gen 20"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "argna"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes units of measurement. Evidence : "adi 10 k"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes graphical emojis. Evidence : " 🤔"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "mt enagmn"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes graphical emojis. Evidence : " 😃"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "hambwmu"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "dnganna"</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains handles or online identifiers. Evidence : "www.google.com"</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains handles or online identifiers.Evidence : "https://pshycolab.com"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "e eka"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "udauk"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "nymayi"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "mn"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns.  Evidence : "wisdewi"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes units of measurement.  Evidence : "Liter"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns.  Evidence : "Liter"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes date information.  Evidence : "2026 | 04 | 26 "</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes date information.  Evidence : "May 12"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns.  Evidence : "tawitra"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes time-related formats.  Evidence : "8.30 a.m"</t>
+  </si>
+  <si>
+    <t>Rationale: The input mentions currency or monetary values. Evidence : "Rs 1500/="</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "Ekkaka"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence " mama"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "yakda"</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains a specific person's name. Evidence : "nipunika"</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains a specific person's name.Evidence : "Nimale"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes names of specific locations. Evidence : "Colombo"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "dawswal"</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes names of specific locations. Evidence : "Kandy"</t>
+  </si>
+  <si>
+    <t>Rationale: The input uses non-standard or varied spelling patterns. Evidence : "awth"</t>
+  </si>
+  <si>
+    <t>Rationale: Shortened English word forms are used. Evidence : "Ad"</t>
+  </si>
+  <si>
+    <t>Rationale: Shortened English word forms are used. Evidence : "Uni"</t>
+  </si>
+  <si>
+    <t>aththatama ewale eyaa hasirunu widiha lol</t>
+  </si>
+  <si>
+    <t>ඇත්තටම ඒවලේ එයා හැසිරුණු විදිහ LOL</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes common English abbreviations or acronyms. Evidence : " lol"</t>
   </si>
 </sst>
 </file>
@@ -1051,7 +1165,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -1070,7 +1184,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>13</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1084,10 +1198,10 @@
         <v>14</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -1106,7 +1220,7 @@
         <v>12</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>13</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1120,7 +1234,7 @@
         <v>14</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>15</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1142,7 +1256,7 @@
         <v>22</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>23</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1156,7 +1270,7 @@
         <v>14</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>15</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1192,7 +1306,7 @@
         <v>14</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>15</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1228,7 +1342,7 @@
         <v>14</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>15</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1239,7 +1353,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>34</v>
@@ -1264,7 +1378,7 @@
         <v>14</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>15</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1289,7 +1403,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1300,7 +1414,7 @@
         <v>14</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>15</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1336,7 +1450,7 @@
         <v>14</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>15</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1372,7 +1486,7 @@
         <v>14</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>15</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1408,7 +1522,7 @@
         <v>14</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>15</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1841,7 +1955,7 @@
         <v>28</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>87</v>
@@ -2046,7 +2160,7 @@
         <v>108</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>109</v>
+        <v>246</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2065,16 +2179,16 @@
     </row>
     <row r="60" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>111</v>
+        <v>244</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>112</v>
+        <v>245</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
@@ -2082,29 +2196,29 @@
         <v>108</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>109</v>
+        <v>246</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
       <c r="G61" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>117</v>
+        <v>243</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2123,46 +2237,46 @@
     </row>
     <row r="63" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
       <c r="G63" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>117</v>
+        <v>242</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
       <c r="G64" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>124</v>
+        <v>240</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2176,29 +2290,29 @@
         <v>14</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>15</v>
+        <v>241</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
       <c r="G66" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>124</v>
+        <v>238</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2212,51 +2326,51 @@
         <v>14</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>15</v>
+        <v>239</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>132</v>
+        <v>237</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
       <c r="G69" s="2" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>132</v>
+        <v>236</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2275,24 +2389,24 @@
     </row>
     <row r="71" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
       <c r="G71" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2306,7 +2420,7 @@
         <v>14</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>15</v>
+        <v>235</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2325,24 +2439,24 @@
     </row>
     <row r="74" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
       <c r="G74" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2356,29 +2470,29 @@
         <v>14</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>15</v>
+        <v>234</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
       <c r="G76" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2392,51 +2506,51 @@
         <v>14</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>15</v>
+        <v>233</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
       <c r="G79" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>156</v>
+        <v>231</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2455,24 +2569,24 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
       <c r="G81" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2486,29 +2600,29 @@
         <v>14</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
       <c r="G83" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>164</v>
+        <v>228</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -2527,46 +2641,46 @@
     </row>
     <row r="85" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="H85" s="2" t="s">
-        <v>164</v>
+        <v>229</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
       <c r="G86" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2580,7 +2694,7 @@
         <v>14</v>
       </c>
       <c r="H87" s="2" t="s">
-        <v>15</v>
+        <v>227</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
@@ -2599,24 +2713,24 @@
     </row>
     <row r="89" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
       <c r="G89" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>172</v>
+        <v>226</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2635,24 +2749,24 @@
     </row>
     <row r="91" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
       <c r="G91" s="2" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2666,7 +2780,7 @@
         <v>14</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>15</v>
+        <v>225</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
@@ -2685,24 +2799,24 @@
     </row>
     <row r="94" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
       <c r="G94" s="2" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2716,29 +2830,29 @@
         <v>14</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>15</v>
+        <v>221</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
       <c r="G96" s="2" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>188</v>
+        <v>220</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2752,29 +2866,29 @@
         <v>14</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>15</v>
+        <v>218</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B98" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
       <c r="G98" s="2" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>188</v>
+        <v>219</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2788,29 +2902,29 @@
         <v>14</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B100" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
       <c r="G100" s="2" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="H100" s="2" t="s">
-        <v>196</v>
+        <v>216</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2824,29 +2938,29 @@
         <v>14</v>
       </c>
       <c r="H101" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="E102" s="3"/>
       <c r="F102" s="3"/>
       <c r="G102" s="2" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="H102" s="2" t="s">
-        <v>196</v>
+        <v>214</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2860,7 +2974,7 @@
         <v>14</v>
       </c>
       <c r="H103" s="2" t="s">
-        <v>15</v>
+        <v>215</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
@@ -2893,24 +3007,24 @@
     </row>
     <row r="106" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="E106" s="3"/>
       <c r="F106" s="3"/>
       <c r="G106" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H106" s="2" t="s">
-        <v>172</v>
+        <v>213</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2924,7 +3038,7 @@
         <v>14</v>
       </c>
       <c r="H107" s="2" t="s">
-        <v>15</v>
+        <v>212</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
@@ -2943,24 +3057,24 @@
     </row>
     <row r="109" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="E109" s="3"/>
       <c r="F109" s="3"/>
       <c r="G109" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="H109" s="2" t="s">
-        <v>140</v>
+        <v>211</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2974,11 +3088,257 @@
         <v>14</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>15</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="270">
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="D61:D62"/>
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="C94:C95"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="D100:D101"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="E106:E108"/>
+    <mergeCell ref="E74:E75"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="F94:F95"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="E76:E77"/>
+    <mergeCell ref="E89:E90"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="E44:E46"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="E71:E73"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="E51:E53"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="F64:F65"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="F51:F53"/>
+    <mergeCell ref="D98:D99"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="F98:F99"/>
+    <mergeCell ref="D41:D43"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="F41:F43"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="C98:C99"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="C51:C53"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="E86:E88"/>
+    <mergeCell ref="A54:A55"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="E58:E59"/>
+    <mergeCell ref="C71:C73"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="A106:A108"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="C100:C101"/>
+    <mergeCell ref="C106:C108"/>
+    <mergeCell ref="C109:C110"/>
+    <mergeCell ref="A74:A75"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D44:D46"/>
+    <mergeCell ref="F44:F46"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="A89:A90"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A76:A77"/>
+    <mergeCell ref="E54:E55"/>
+    <mergeCell ref="C76:C77"/>
+    <mergeCell ref="F100:F101"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="F109:F110"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="F25:F27"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="F96:F97"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="D79:D80"/>
+    <mergeCell ref="D86:D88"/>
+    <mergeCell ref="F86:F88"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="D94:D95"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="A94:A95"/>
+    <mergeCell ref="D106:D108"/>
+    <mergeCell ref="F106:F108"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="F74:F75"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B91:B93"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="D83:D84"/>
+    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="D71:D73"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="F89:F90"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="D76:D77"/>
+    <mergeCell ref="F76:F77"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D51:D53"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="F66:F67"/>
+    <mergeCell ref="C86:C88"/>
+    <mergeCell ref="E94:E95"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B86:B88"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="D91:D93"/>
+    <mergeCell ref="F91:F93"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="A58:A59"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E91:E93"/>
+    <mergeCell ref="E25:E27"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="F56:F57"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="F58:F59"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="A98:A99"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="E96:E97"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="B100:B101"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="B109:B110"/>
+    <mergeCell ref="F31:F33"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="D109:D110"/>
+    <mergeCell ref="F71:F73"/>
+    <mergeCell ref="B96:B97"/>
+    <mergeCell ref="D96:D97"/>
+    <mergeCell ref="C89:C90"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A91:A93"/>
+    <mergeCell ref="E98:E99"/>
+    <mergeCell ref="F28:F30"/>
+    <mergeCell ref="C91:C93"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="B39:B40"/>
     <mergeCell ref="B106:B108"/>
     <mergeCell ref="C61:C62"/>
     <mergeCell ref="E61:E62"/>
@@ -3003,252 +3363,6 @@
     <mergeCell ref="A64:A65"/>
     <mergeCell ref="D69:D70"/>
     <mergeCell ref="A86:A88"/>
-    <mergeCell ref="A98:A99"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="E96:E97"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="B100:B101"/>
-    <mergeCell ref="F22:F24"/>
-    <mergeCell ref="B109:B110"/>
-    <mergeCell ref="F31:F33"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="D109:D110"/>
-    <mergeCell ref="F71:F73"/>
-    <mergeCell ref="B96:B97"/>
-    <mergeCell ref="D96:D97"/>
-    <mergeCell ref="C89:C90"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A91:A93"/>
-    <mergeCell ref="E98:E99"/>
-    <mergeCell ref="F28:F30"/>
-    <mergeCell ref="C91:C93"/>
-    <mergeCell ref="E41:E43"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B86:B88"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="D91:D93"/>
-    <mergeCell ref="F91:F93"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="A83:A84"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="A58:A59"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E91:E93"/>
-    <mergeCell ref="E25:E27"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="F56:F57"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="F58:F59"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="D71:D73"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="F89:F90"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="D76:D77"/>
-    <mergeCell ref="F76:F77"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D51:D53"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="F66:F67"/>
-    <mergeCell ref="C86:C88"/>
-    <mergeCell ref="E94:E95"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="A94:A95"/>
-    <mergeCell ref="D106:D108"/>
-    <mergeCell ref="F106:F108"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="F74:F75"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="B98:B99"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B91:B93"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="D83:D84"/>
-    <mergeCell ref="F34:F36"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="F109:F110"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="F25:F27"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="F96:F97"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="D79:D80"/>
-    <mergeCell ref="D86:D88"/>
-    <mergeCell ref="F86:F88"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="A25:A27"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="C74:C75"/>
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="D94:D95"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="A106:A108"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="C100:C101"/>
-    <mergeCell ref="C106:C108"/>
-    <mergeCell ref="C109:C110"/>
-    <mergeCell ref="A74:A75"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="A56:A57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D44:D46"/>
-    <mergeCell ref="F44:F46"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="A89:A90"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A76:A77"/>
-    <mergeCell ref="E54:E55"/>
-    <mergeCell ref="C76:C77"/>
-    <mergeCell ref="F100:F101"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A79:A80"/>
-    <mergeCell ref="A61:A62"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="E86:E88"/>
-    <mergeCell ref="A54:A55"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="F54:F55"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="E58:E59"/>
-    <mergeCell ref="C71:C73"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="F51:F53"/>
-    <mergeCell ref="D98:D99"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="F98:F99"/>
-    <mergeCell ref="D41:D43"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="F41:F43"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C98:C99"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="E71:E73"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="E51:E53"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="F64:F65"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="E106:E108"/>
-    <mergeCell ref="E74:E75"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="F94:F95"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="E76:E77"/>
-    <mergeCell ref="E89:E90"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="E44:E46"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="C51:C53"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="D61:D62"/>
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="D100:D101"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>